<commit_message>
Continued working on some testing cases. Only few remaining now.
</commit_message>
<xml_diff>
--- a/Tests/CSCS_Frontend_Test_Suite.xlsx
+++ b/Tests/CSCS_Frontend_Test_Suite.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/achrafcheniti/Documents/Summer_2026/COMP 353/cscs-db-353/Tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31931B10-26E6-4E42-81B7-7354E0757C3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A3F7492-9D7C-EF42-8084-6C75FF872B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16100" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="226">
   <si>
     <t>CSCS Main Project — Frontend Constraint Test Plan</t>
   </si>
@@ -789,6 +789,28 @@
   </si>
   <si>
     <t>Works fine</t>
+  </si>
+  <si>
+    <t>Record added successfully</t>
+  </si>
+  <si>
+    <t>16-08-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both team formations in a session must be the same category (Boys or Girls).
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A session can contain exactly two team formations; a third formation is not allowed.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Club member location does not match the team formation location.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Club member gender does not match the team formation category.
+</t>
   </si>
 </sst>
 </file>
@@ -2051,11 +2073,17 @@
         <v>132</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
-      <c r="M16" s="8"/>
+        <v>201</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="L16" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="M16" s="8" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="17" spans="1:13" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
@@ -2086,11 +2114,17 @@
         <v>137</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="8"/>
+        <v>201</v>
+      </c>
+      <c r="K17" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="M17" s="8" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="18" spans="1:13" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
@@ -2121,11 +2155,17 @@
         <v>141</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
-      <c r="M18" s="8"/>
+        <v>201</v>
+      </c>
+      <c r="K18" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="L18" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="M18" s="8" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="19" spans="1:13" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
@@ -2156,11 +2196,17 @@
         <v>146</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
-      <c r="M19" s="8"/>
+        <v>201</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L19" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="20" spans="1:13" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
@@ -2191,11 +2237,17 @@
         <v>153</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="8"/>
+        <v>201</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="L20" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="M20" s="8" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="21" spans="1:13" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
@@ -2226,13 +2278,19 @@
         <v>158</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
-      <c r="M21" s="8"/>
-    </row>
-    <row r="22" spans="1:13" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+        <v>201</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="L21" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="M21" s="8" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="70" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>159</v>
       </c>
@@ -2688,7 +2746,7 @@
       </c>
       <c r="C8" s="12">
         <f>COUNTIFS('Test Cases'!$B$2:$B$29,A8,'Test Cases'!$J$2:$J$29,"Passed")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D8" s="12">
         <f>COUNTIFS('Test Cases'!$B$2:$B$29,A8,'Test Cases'!$J$2:$J$29,"Failed")</f>
@@ -2700,7 +2758,7 @@
       </c>
       <c r="F8" s="12">
         <f>COUNTIFS('Test Cases'!$B$2:$B$29,A8,'Test Cases'!$J$2:$J$29,"Not Run")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -2713,7 +2771,7 @@
       </c>
       <c r="C9" s="12">
         <f>COUNTIFS('Test Cases'!$B$2:$B$29,A9,'Test Cases'!$J$2:$J$29,"Passed")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D9" s="12">
         <f>COUNTIFS('Test Cases'!$B$2:$B$29,A9,'Test Cases'!$J$2:$J$29,"Failed")</f>
@@ -2725,7 +2783,7 @@
       </c>
       <c r="F9" s="12">
         <f>COUNTIFS('Test Cases'!$B$2:$B$29,A9,'Test Cases'!$J$2:$J$29,"Not Run")</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -2763,7 +2821,7 @@
       </c>
       <c r="C11" s="14">
         <f>SUM(C4:C10)</f>
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D11" s="14">
         <f>SUM(D4:D10)</f>
@@ -2775,7 +2833,7 @@
       </c>
       <c r="F11" s="14">
         <f>SUM(F4:F10)</f>
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -2784,7 +2842,7 @@
       </c>
       <c r="B13" s="15">
         <f>IFERROR(C11/(C11+D11+E11),"n/a")</f>
-        <v>0.7142857142857143</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>